<commit_message>
Add SNDK and AAPL to watchlist
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/watchlist.xlsx
+++ b/watchlist.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Watchlist" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Watchlist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -579,6 +579,30 @@
       <c r="B11" t="inlineStr">
         <is>
           <t>edge / on-device AI</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NAND flash / storage (SanDisk)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>consumer devices and services</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Group Cross-Company Summary and Company Detail by watchlist category
Expand watchlist to 32 AI-supply-chain tickers organized into 6 categories
(accelerators, hyperscalers, memory, fabs/tools/EDA, power/systems, and
interconnect). The report now renders a separate table/card group per
category when the watchlist has a category column, falling back to the
previous flat layout when it doesn't.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/watchlist.xlsx
+++ b/watchlist.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -461,6 +461,11 @@
           <t>note</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -470,31 +475,46 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>GPUs - dominant AI accelerator</t>
+          <t>Merchant GPUs + CUDA software moat</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Accelerators &amp; compute silicon</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Instinct accelerators</t>
+          <t>Custom ASICs (XPUs) for hyperscalers + networking silicon</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Accelerators &amp; compute silicon</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>custom accelerators, networking</t>
+          <t>Instinct MI GPUs, the main merchant alternative to NVDA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Accelerators &amp; compute silicon</t>
         </is>
       </c>
     </row>
@@ -506,103 +526,488 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>custom AI silicon, interconnect</t>
+          <t>Custom AI silicon, optical DSP, interconnect</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Accelerators &amp; compute silicon</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EUV lithography</t>
+          <t>CPU architecture IP licensed into AI systems</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Accelerators &amp; compute silicon</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>high-bandwidth memory</t>
+          <t>Gaudi accelerators, foundry</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Accelerators &amp; compute silicon</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TPUs - note: ads/cloud driven, not a pure chip name</t>
+          <t>Edge / on-device AI</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Accelerators &amp; compute silicon</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>INTC</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gaudi, foundry</t>
+          <t>On-device AI silicon; consumer demand signal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Hyperscalers &amp; end demand</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>fabricates most leading-edge AI chips</t>
+          <t>TPUs, the deepest in-house accelerator program</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Hyperscalers &amp; end demand</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>edge / on-device AI</t>
+          <t>Trainium / Inferentia + AWS capacity</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Hyperscalers &amp; end demand</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>NAND flash / storage (SanDisk)</t>
+          <t>Maia accelerators + Azure</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Hyperscalers &amp; end demand</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>consumer devices and services</t>
+          <t>MTIA silicon; among the largest GPU buyers</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Hyperscalers &amp; end demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>MU</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HBM and DRAM, the memory bottleneck</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Memory &amp; storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SKHY</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SK Hynix ADR, HBM share leader</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Memory &amp; storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SNDK</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NAND flash</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Memory &amp; storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WDC</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>High-capacity HDD for data-centre storage</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Memory &amp; storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Foundry, manufactures nearly every leading AI chip</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Fabs, tools &amp; EDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ASML</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>EUV lithography, effectively a monopoly</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Fabs, tools &amp; EDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AMAT</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Deposition and etch</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Fabs, tools &amp; EDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>LRCX</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Etch and deposition, key to HBM stacking</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Fabs, tools &amp; EDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>KLAC</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Process control and inspection</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Fabs, tools &amp; EDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Chip test, including HBM</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Fabs, tools &amp; EDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CDNS</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>EDA design software</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Fabs, tools &amp; EDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SNPS</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>EDA plus silicon IP</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Fabs, tools &amp; EDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Power and thermal for high-density racks</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Power, systems &amp; neoclouds</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SMCI</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>AI server and rack integration</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Power, systems &amp; neoclouds</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>AI servers at enterprise scale</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Power, systems &amp; neoclouds</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>CRWV</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>GPU cloud (neocloud)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Power, systems &amp; neoclouds</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Data-centre hosting for HPC</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Power, systems &amp; neoclouds</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ALAB</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>PCIe retimers and fabric, inside the rack</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Interconnect &amp; networking</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>CRDO</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Active electrical cables, SerDes</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Interconnect &amp; networking</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ANET</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Ethernet switching, between racks</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Interconnect &amp; networking</t>
         </is>
       </c>
     </row>

</xml_diff>